<commit_message>
cluster analysis upd. (prop visnorm)
</commit_message>
<xml_diff>
--- a/clustering/8 subclusters (factoriescap_s (costs) 0 prop visnorm).xlsx
+++ b/clustering/8 subclusters (factoriescap_s (costs) 0 prop visnorm).xlsx
@@ -43,11 +43,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0000%"/>
-    <numFmt numFmtId="165" formatCode="0.000%"/>
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -76,6 +75,13 @@
       <charset val="204"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="204"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -86,7 +92,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FF00B050"/>
+        <fgColor rgb="FF92D050"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -119,7 +125,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -127,22 +133,25 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="2" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
@@ -159,6 +168,55 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>19050</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>323992</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Рисунок 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="6000750" y="19050"/>
+          <a:ext cx="5315092" cy="3267075"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -446,13 +504,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.5703125" customWidth="1"/>
-    <col min="3" max="3" width="15.7109375" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" customWidth="1"/>
+    <col min="2" max="2" width="19.7109375" customWidth="1"/>
+    <col min="3" max="3" width="19.42578125" customWidth="1"/>
+    <col min="4" max="4" width="17.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
@@ -476,152 +534,152 @@
       <c r="A2" s="2">
         <v>0</v>
       </c>
-      <c r="B2" s="3">
-        <v>494847.27047901019</v>
-      </c>
-      <c r="C2" s="4">
-        <v>2.3614395320195121E-3</v>
-      </c>
-      <c r="D2" s="4">
-        <v>6.8755236621103461E-4</v>
-      </c>
-      <c r="E2" s="4">
-        <v>7.0305306132489799E-4</v>
+      <c r="B2" s="2">
+        <v>513836.84339999908</v>
+      </c>
+      <c r="C2" s="7">
+        <v>3.2040540384835128E-3</v>
+      </c>
+      <c r="D2" s="7">
+        <v>3.6027102385206792E-3</v>
+      </c>
+      <c r="E2" s="7">
+        <v>1.382769540800156E-3</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>0</v>
       </c>
-      <c r="B3" s="3">
-        <v>5137890.7677814802</v>
-      </c>
-      <c r="C3" s="4">
-        <v>5.8827587026286836E-3</v>
-      </c>
-      <c r="D3" s="4">
-        <v>5.7172167306981849E-3</v>
-      </c>
-      <c r="E3" s="4">
-        <v>3.2578372481786981E-3</v>
+      <c r="B3" s="2">
+        <v>4568912.8562746271</v>
+      </c>
+      <c r="C3" s="7">
+        <v>3.043993965460933E-3</v>
+      </c>
+      <c r="D3" s="7">
+        <v>7.1739340238030731E-3</v>
+      </c>
+      <c r="E3" s="7">
+        <v>1.546349960720892E-3</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>1</v>
       </c>
-      <c r="B4" s="3">
-        <v>696644.36444999697</v>
-      </c>
-      <c r="C4" s="4">
-        <v>3.8865980051246071E-3</v>
-      </c>
-      <c r="D4" s="4">
-        <v>5.2561440081365512E-2</v>
-      </c>
-      <c r="E4" s="4">
-        <v>7.8647681063912065E-4</v>
+      <c r="B4" s="2">
+        <v>1169072.66356</v>
+      </c>
+      <c r="C4" s="7">
+        <v>1.4231071957161039E-2</v>
+      </c>
+      <c r="D4" s="7">
+        <v>9.5124144125518263E-3</v>
+      </c>
+      <c r="E4" s="7">
+        <v>8.5056280961609276E-3</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>1</v>
       </c>
-      <c r="B5" s="3">
-        <v>1731990.4654999969</v>
-      </c>
-      <c r="C5" s="4">
-        <v>7.6474050544495797E-3</v>
-      </c>
-      <c r="D5" s="4">
-        <v>8.2459680283814354E-2</v>
-      </c>
-      <c r="E5" s="4">
-        <v>1.6986052410676159E-3</v>
+      <c r="B5" s="2">
+        <v>3901118.3733799988</v>
+      </c>
+      <c r="C5" s="7">
+        <v>1.4477852829466941E-2</v>
+      </c>
+      <c r="D5" s="7">
+        <v>1.230742909455026E-2</v>
+      </c>
+      <c r="E5" s="7">
+        <v>9.9750357519423107E-3</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>2</v>
       </c>
-      <c r="B6" s="3">
-        <v>954612.73294285475</v>
-      </c>
-      <c r="C6" s="4">
-        <v>1.2208530216390659E-2</v>
-      </c>
-      <c r="D6" s="4">
-        <v>3.9409780369331817E-3</v>
-      </c>
-      <c r="E6" s="4">
-        <v>1.1826477366159759E-3</v>
+      <c r="B6" s="2">
+        <v>476236.26529166597</v>
+      </c>
+      <c r="C6" s="7">
+        <v>8.2923793187854276E-3</v>
+      </c>
+      <c r="D6" s="7">
+        <v>3.2726079522927549E-3</v>
+      </c>
+      <c r="E6" s="7">
+        <v>1.4432721746225759E-3</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>2</v>
       </c>
-      <c r="B7" s="3">
-        <v>3920985.008428568</v>
-      </c>
-      <c r="C7" s="4">
-        <v>1.752384975236905E-2</v>
-      </c>
-      <c r="D7" s="4">
-        <v>1.501027826977259E-2</v>
-      </c>
-      <c r="E7" s="4">
-        <v>1.3185364916054281E-2</v>
+      <c r="B7" s="2">
+        <v>2138222.5147666661</v>
+      </c>
+      <c r="C7" s="7">
+        <v>8.0285881209146755E-3</v>
+      </c>
+      <c r="D7" s="7">
+        <v>3.5810411504599718E-3</v>
+      </c>
+      <c r="E7" s="7">
+        <v>2.3276246028009909E-3</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>3</v>
       </c>
-      <c r="B8" s="3">
-        <v>1078041.1206333309</v>
-      </c>
-      <c r="C8" s="4">
-        <v>2.6867632207750081E-3</v>
-      </c>
-      <c r="D8" s="4">
-        <v>1.6585148722047159E-2</v>
-      </c>
-      <c r="E8" s="4">
-        <v>7.2172550955266156E-4</v>
+      <c r="B8" s="2">
+        <v>782813.64053333236</v>
+      </c>
+      <c r="C8" s="7">
+        <v>4.3586102450761423E-3</v>
+      </c>
+      <c r="D8" s="7">
+        <v>6.1807776562022222E-2</v>
+      </c>
+      <c r="E8" s="7">
+        <v>1.25370625976207E-3</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>3</v>
       </c>
-      <c r="B9" s="3">
-        <v>14221383.2367</v>
-      </c>
-      <c r="C9" s="4">
-        <v>5.8112421781721874E-3</v>
-      </c>
-      <c r="D9" s="4">
-        <v>2.9819087249808959E-2</v>
-      </c>
-      <c r="E9" s="4">
-        <v>1.1866108407711949E-2</v>
+      <c r="B9" s="2">
+        <v>3167644.9749333318</v>
+      </c>
+      <c r="C9" s="7">
+        <v>6.0248174940261698E-3</v>
+      </c>
+      <c r="D9" s="7">
+        <v>5.837911999034965E-2</v>
+      </c>
+      <c r="E9" s="7">
+        <v>1.2723893622083361E-3</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="1" t="s">
+      <c r="A12" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D12" s="1" t="s">
+      <c r="D12" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" s="3" t="s">
         <v>4</v>
       </c>
     </row>
@@ -634,386 +692,206 @@
       <c r="A14" s="2">
         <v>0</v>
       </c>
-      <c r="B14" s="5">
+      <c r="B14" s="4">
         <f>B3/B2</f>
-        <v>10.38278085844148</v>
-      </c>
-      <c r="C14" s="3">
+        <v>8.8917579869179058</v>
+      </c>
+      <c r="C14" s="5">
         <f>C3/C2</f>
-        <v>2.4911748206390558</v>
+        <v>0.95004451513610033</v>
       </c>
       <c r="D14" s="6">
         <f t="shared" ref="D14:E20" si="0">D3/D2</f>
-        <v>8.3153182385287074</v>
-      </c>
-      <c r="E14" s="3">
+        <v>1.9912603425883026</v>
+      </c>
+      <c r="E14" s="6">
         <f t="shared" si="0"/>
-        <v>4.6338426320757771</v>
+        <v>1.1182991200587757</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>1</v>
       </c>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="5"/>
+      <c r="E15" s="5"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>1</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="5">
         <f>B5/B4</f>
-        <v>2.4861903058204011</v>
-      </c>
-      <c r="C16" s="3">
+        <v>3.3369340460844525</v>
+      </c>
+      <c r="C16" s="6">
         <f>C5/C4</f>
-        <v>1.9676346883228533</v>
-      </c>
-      <c r="D16" s="3">
+        <v>1.0173409897053975</v>
+      </c>
+      <c r="D16" s="6">
         <f t="shared" si="0"/>
-        <v>1.5688246013839449</v>
+        <v>1.2938281030219156</v>
       </c>
       <c r="E16" s="6">
         <f t="shared" si="0"/>
-        <v>2.1597651934419595</v>
+        <v>1.1727571014355318</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="2">
         <v>2</v>
       </c>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="5"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="2">
         <v>2</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="5">
         <f>B7/B6</f>
-        <v>4.1074090813151631</v>
-      </c>
-      <c r="C18" s="3">
+        <v>4.4898355513877837</v>
+      </c>
+      <c r="C18" s="5">
         <f>C7/C6</f>
-        <v>1.4353775140632625</v>
+        <v>0.96818872030212566</v>
       </c>
       <c r="D18" s="6">
         <f t="shared" si="0"/>
-        <v>3.8087698355846191</v>
-      </c>
-      <c r="E18" s="3">
+        <v>1.0942469133680164</v>
+      </c>
+      <c r="E18" s="6">
         <f t="shared" si="0"/>
-        <v>11.149021393118156</v>
+        <v>1.6127412720401668</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="2">
         <v>3</v>
       </c>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="2">
         <v>3</v>
       </c>
-      <c r="B20" s="3">
+      <c r="B20" s="5">
         <f>B9/B8</f>
-        <v>13.191874562581786</v>
-      </c>
-      <c r="C20" s="3">
+        <v>4.046486687144605</v>
+      </c>
+      <c r="C20" s="6">
         <f>C9/C8</f>
-        <v>2.1629156351544481</v>
-      </c>
-      <c r="D20" s="3">
+        <v>1.3822794779212748</v>
+      </c>
+      <c r="D20" s="4">
         <f t="shared" si="0"/>
-        <v>1.7979390929530532</v>
-      </c>
-      <c r="E20" s="6">
+        <v>0.94452710059498712</v>
+      </c>
+      <c r="E20" s="4">
         <f t="shared" si="0"/>
-        <v>16.441303862276914</v>
+        <v>1.0149022965314154</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A23" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
-        <v>5</v>
+      <c r="A24" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B24" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="E24" s="3" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
+      <c r="A25" s="2">
         <v>0</v>
       </c>
-      <c r="B25" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E25" s="1" t="s">
-        <v>4</v>
+      <c r="B25" s="8">
+        <v>1039934.962199999</v>
+      </c>
+      <c r="C25" s="7">
+        <v>2.9568939200096209E-3</v>
+      </c>
+      <c r="D25" s="7">
+        <v>2.5765194972923872E-3</v>
+      </c>
+      <c r="E25" s="7">
+        <v>1.0641046375700089E-3</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="2">
-        <v>0</v>
-      </c>
-      <c r="B26" s="2">
-        <v>993615.17969999847</v>
-      </c>
-      <c r="C26" s="8">
-        <v>3.5324517025561351E-3</v>
-      </c>
-      <c r="D26" s="8">
-        <v>1.673724645056331E-3</v>
-      </c>
-      <c r="E26" s="8">
-        <v>1.197008269244631E-3</v>
+        <v>1</v>
+      </c>
+      <c r="B26" s="8">
+        <v>2686820.6399999992</v>
+      </c>
+      <c r="C26" s="7">
+        <v>1.5160173283880741E-2</v>
+      </c>
+      <c r="D26" s="7">
+        <v>9.6489513212821947E-3</v>
+      </c>
+      <c r="E26" s="7">
+        <v>2.9649214976894202E-3</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="2">
-        <v>1</v>
-      </c>
-      <c r="B27" s="2">
-        <v>1186586.399999998</v>
-      </c>
-      <c r="C27" s="8">
-        <v>4.4260834436022859E-3</v>
-      </c>
-      <c r="D27" s="8">
-        <v>6.3756715528644717E-2</v>
-      </c>
-      <c r="E27" s="8">
-        <v>1.053600347757846E-3</v>
+        <v>2</v>
+      </c>
+      <c r="B27" s="8">
+        <v>1039044.479999998</v>
+      </c>
+      <c r="C27" s="7">
+        <v>7.6216305472655774E-3</v>
+      </c>
+      <c r="D27" s="7">
+        <v>1.365428704605655E-3</v>
+      </c>
+      <c r="E27" s="7">
+        <v>1.2338530084869341E-3</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="2">
-        <v>2</v>
-      </c>
-      <c r="B28" s="2">
-        <v>2325159.738599997</v>
-      </c>
-      <c r="C28" s="8">
-        <v>1.4495460515713651E-2</v>
-      </c>
-      <c r="D28" s="8">
-        <v>8.570628609736031E-3</v>
-      </c>
-      <c r="E28" s="8">
-        <v>1.9695490726824071E-3</v>
-      </c>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="2">
         <v>3</v>
       </c>
-      <c r="B29" s="2">
-        <v>2422113.7299999991</v>
-      </c>
-      <c r="C29" s="8">
-        <v>4.0288180097590017E-3</v>
-      </c>
-      <c r="D29" s="8">
-        <v>2.1392756463782959E-2</v>
-      </c>
-      <c r="E29" s="8">
-        <v>1.064104637569974E-3</v>
+      <c r="B28" s="8">
+        <v>1191650.4643999999</v>
+      </c>
+      <c r="C28" s="7">
+        <v>4.3807805911778722E-3</v>
+      </c>
+      <c r="D28" s="7">
+        <v>5.4076639058523807E-2</v>
+      </c>
+      <c r="E28" s="7">
+        <v>1.152625659984912E-3</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B3">
-    <cfRule type="colorScale" priority="24">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C3">
-    <cfRule type="colorScale" priority="23">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D3">
-    <cfRule type="colorScale" priority="22">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E2:E3">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B4:B5">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B6:B7">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B8:B9">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C4:C5">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D4:D5">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E4:E5">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C6:C7">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D6:D7">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E6:E7">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C8:C9">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="D8:D9">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E8:E9">
-    <cfRule type="colorScale" priority="9">
+  <conditionalFormatting sqref="B2:B9">
+    <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1025,7 +903,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C2:C9">
-    <cfRule type="colorScale" priority="8">
+    <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1037,7 +915,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D2:D9">
-    <cfRule type="colorScale" priority="7">
+    <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -1049,18 +927,6 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E2:E9">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="FFF8696B"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B9">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -1072,7 +938,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B26:B29">
+  <conditionalFormatting sqref="B25:B28">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1084,7 +950,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C26:C29">
+  <conditionalFormatting sqref="C25:C28">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1096,7 +962,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D26:D29">
+  <conditionalFormatting sqref="D25:D28">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1108,7 +974,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E26:E29">
+  <conditionalFormatting sqref="E25:E28">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1122,5 +988,6 @@
   </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>